<commit_message>
updated index rmd to include auto summary table
</commit_message>
<xml_diff>
--- a/data/input/mgt_targets.xlsx
+++ b/data/input/mgt_targets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\SRAFS\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2362FA7-A0BC-44A2-A206-98358A0DD00A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A6B8FA6-D8D8-4AD3-BDB9-86790E19BC51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Goals and Thresholds" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2026" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2303" uniqueCount="110">
   <si>
     <t xml:space="preserve">Total </t>
   </si>
@@ -483,6 +483,15 @@
   </si>
   <si>
     <t>Hells Canyon</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>Extirpated</t>
+  </si>
+  <si>
+    <t>Extant</t>
   </si>
 </sst>
 </file>
@@ -2168,7 +2177,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H277"/>
+  <dimension ref="A1:I277"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" bestFit="1" customWidth="1"/>
@@ -2178,10 +2187,11 @@
     <col min="5" max="5" width="20.5703125" customWidth="1"/>
     <col min="6" max="6" width="21.5703125" customWidth="1"/>
     <col min="7" max="7" width="16.85546875" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" customWidth="1"/>
+    <col min="8" max="8" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>30</v>
       </c>
@@ -2206,8 +2216,11 @@
       <c r="H1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2232,8 +2245,11 @@
       <c r="H2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2258,8 +2274,11 @@
       <c r="H3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2284,8 +2303,11 @@
       <c r="H4" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2310,8 +2332,11 @@
       <c r="H5" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2336,8 +2361,11 @@
       <c r="H6" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2362,8 +2390,11 @@
       <c r="H7" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2388,8 +2419,11 @@
       <c r="H8" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2414,8 +2448,11 @@
       <c r="H9" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2440,8 +2477,11 @@
       <c r="H10" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2466,8 +2506,11 @@
       <c r="H11" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2492,8 +2535,11 @@
       <c r="H12" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2518,8 +2564,11 @@
       <c r="H13" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2544,8 +2593,11 @@
       <c r="H14" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I14" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>3</v>
       </c>
@@ -2570,8 +2622,11 @@
       <c r="H15" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I15" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>3</v>
       </c>
@@ -2596,8 +2651,11 @@
       <c r="H16" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I16" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -2622,8 +2680,11 @@
       <c r="H17" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I17" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -2648,8 +2709,11 @@
       <c r="H18" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>3</v>
       </c>
@@ -2674,8 +2738,11 @@
       <c r="H19" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I19" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>3</v>
       </c>
@@ -2700,8 +2767,11 @@
       <c r="H20" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I20" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -2726,8 +2796,11 @@
       <c r="H21" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I21" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>3</v>
       </c>
@@ -2752,8 +2825,11 @@
       <c r="H22" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I22" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>3</v>
       </c>
@@ -2778,8 +2854,11 @@
       <c r="H23" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I23" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>3</v>
       </c>
@@ -2804,8 +2883,11 @@
       <c r="H24" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I24" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>3</v>
       </c>
@@ -2830,8 +2912,11 @@
       <c r="H25" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I25" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>3</v>
       </c>
@@ -2856,8 +2941,11 @@
       <c r="H26" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I26" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>3</v>
       </c>
@@ -2882,8 +2970,11 @@
       <c r="H27" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I27" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>3</v>
       </c>
@@ -2908,8 +2999,11 @@
       <c r="H28" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I28" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>3</v>
       </c>
@@ -2934,8 +3028,11 @@
       <c r="H29" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>3</v>
       </c>
@@ -2960,8 +3057,11 @@
       <c r="H30" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I30" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>3</v>
       </c>
@@ -2986,8 +3086,11 @@
       <c r="H31" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I31" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>3</v>
       </c>
@@ -3012,8 +3115,11 @@
       <c r="H32" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I32" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>3</v>
       </c>
@@ -3038,8 +3144,11 @@
       <c r="H33" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I33" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>3</v>
       </c>
@@ -3064,8 +3173,11 @@
       <c r="H34" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I34" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>3</v>
       </c>
@@ -3090,8 +3202,11 @@
       <c r="H35" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I35" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>3</v>
       </c>
@@ -3116,8 +3231,11 @@
       <c r="H36" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I36" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>3</v>
       </c>
@@ -3142,8 +3260,11 @@
       <c r="H37" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I37" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -3168,8 +3289,11 @@
       <c r="H38" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I38" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -3194,8 +3318,11 @@
       <c r="H39" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I39" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -3220,8 +3347,11 @@
       <c r="H40" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I40" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -3246,8 +3376,11 @@
       <c r="H41" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I41" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -3272,8 +3405,11 @@
       <c r="H42" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I42" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -3298,8 +3434,11 @@
       <c r="H43" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I43" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -3324,8 +3463,11 @@
       <c r="H44" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I44" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -3350,8 +3492,11 @@
       <c r="H45" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I45" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -3376,8 +3521,11 @@
       <c r="H46" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I46" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -3402,8 +3550,11 @@
       <c r="H47" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I47" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -3428,8 +3579,11 @@
       <c r="H48" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I48" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -3454,8 +3608,11 @@
       <c r="H49" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I49" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -3480,8 +3637,11 @@
       <c r="H50" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I50" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -3506,8 +3666,11 @@
       <c r="H51" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I51" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -3532,8 +3695,11 @@
       <c r="H52" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I52" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -3558,8 +3724,11 @@
       <c r="H53" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I53" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -3584,8 +3753,11 @@
       <c r="H54" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I54" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -3610,8 +3782,11 @@
       <c r="H55" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I55" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>3</v>
       </c>
@@ -3636,8 +3811,11 @@
       <c r="H56" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I56" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>3</v>
       </c>
@@ -3662,8 +3840,11 @@
       <c r="H57" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I57" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>3</v>
       </c>
@@ -3688,8 +3869,11 @@
       <c r="H58" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I58" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>3</v>
       </c>
@@ -3714,8 +3898,11 @@
       <c r="H59" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I59" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>3</v>
       </c>
@@ -3740,8 +3927,11 @@
       <c r="H60" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I60" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>3</v>
       </c>
@@ -3766,8 +3956,11 @@
       <c r="H61" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I61" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>3</v>
       </c>
@@ -3792,8 +3985,11 @@
       <c r="H62" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I62" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>3</v>
       </c>
@@ -3818,8 +4014,11 @@
       <c r="H63" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I63" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>3</v>
       </c>
@@ -3844,8 +4043,11 @@
       <c r="H64" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I64" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>3</v>
       </c>
@@ -3870,8 +4072,11 @@
       <c r="H65" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I65" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>3</v>
       </c>
@@ -3896,8 +4101,11 @@
       <c r="H66" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I66" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>3</v>
       </c>
@@ -3922,8 +4130,11 @@
       <c r="H67" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I67" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>3</v>
       </c>
@@ -3948,8 +4159,11 @@
       <c r="H68" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I68" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>3</v>
       </c>
@@ -3974,8 +4188,11 @@
       <c r="H69" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I69" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>3</v>
       </c>
@@ -4000,8 +4217,11 @@
       <c r="H70" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I70" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>3</v>
       </c>
@@ -4026,8 +4246,11 @@
       <c r="H71" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I71" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>3</v>
       </c>
@@ -4052,8 +4275,11 @@
       <c r="H72" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I72" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>3</v>
       </c>
@@ -4078,8 +4304,11 @@
       <c r="H73" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I73" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>3</v>
       </c>
@@ -4104,8 +4333,11 @@
       <c r="H74" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I74" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>3</v>
       </c>
@@ -4130,8 +4362,11 @@
       <c r="H75" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I75" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>3</v>
       </c>
@@ -4156,8 +4391,11 @@
       <c r="H76" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I76" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>3</v>
       </c>
@@ -4182,8 +4420,11 @@
       <c r="H77" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I77" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>3</v>
       </c>
@@ -4208,8 +4449,11 @@
       <c r="H78" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I78" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>3</v>
       </c>
@@ -4234,8 +4478,11 @@
       <c r="H79" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I79" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>3</v>
       </c>
@@ -4260,8 +4507,11 @@
       <c r="H80" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I80" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>3</v>
       </c>
@@ -4286,8 +4536,11 @@
       <c r="H81" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I81" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>3</v>
       </c>
@@ -4312,8 +4565,11 @@
       <c r="H82" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I82" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>3</v>
       </c>
@@ -4338,8 +4594,11 @@
       <c r="H83" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I83" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>3</v>
       </c>
@@ -4364,8 +4623,11 @@
       <c r="H84" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I84" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>3</v>
       </c>
@@ -4390,8 +4652,11 @@
       <c r="H85" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I85" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>3</v>
       </c>
@@ -4416,8 +4681,11 @@
       <c r="H86" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I86" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>3</v>
       </c>
@@ -4442,8 +4710,11 @@
       <c r="H87" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I87" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>3</v>
       </c>
@@ -4468,8 +4739,11 @@
       <c r="H88" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I88" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>3</v>
       </c>
@@ -4494,8 +4768,11 @@
       <c r="H89" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I89" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>3</v>
       </c>
@@ -4520,8 +4797,11 @@
       <c r="H90" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I90" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>3</v>
       </c>
@@ -4546,8 +4826,11 @@
       <c r="H91" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I91" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>3</v>
       </c>
@@ -4572,8 +4855,11 @@
       <c r="H92" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I92" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>3</v>
       </c>
@@ -4598,8 +4884,11 @@
       <c r="H93" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I93" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>3</v>
       </c>
@@ -4624,8 +4913,11 @@
       <c r="H94" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I94" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>3</v>
       </c>
@@ -4650,8 +4942,11 @@
       <c r="H95" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I95" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>3</v>
       </c>
@@ -4676,8 +4971,11 @@
       <c r="H96" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I96" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>3</v>
       </c>
@@ -4702,8 +5000,11 @@
       <c r="H97" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I97" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>3</v>
       </c>
@@ -4728,8 +5029,11 @@
       <c r="H98" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I98" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>3</v>
       </c>
@@ -4754,8 +5058,11 @@
       <c r="H99" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I99" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>3</v>
       </c>
@@ -4780,8 +5087,11 @@
       <c r="H100" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I100" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>3</v>
       </c>
@@ -4806,8 +5116,11 @@
       <c r="H101" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I101" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>3</v>
       </c>
@@ -4832,8 +5145,11 @@
       <c r="H102" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I102" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>3</v>
       </c>
@@ -4858,8 +5174,11 @@
       <c r="H103" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I103" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>3</v>
       </c>
@@ -4884,8 +5203,11 @@
       <c r="H104" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I104" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>3</v>
       </c>
@@ -4910,8 +5232,11 @@
       <c r="H105" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I105" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>3</v>
       </c>
@@ -4936,8 +5261,11 @@
       <c r="H106" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I106" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>3</v>
       </c>
@@ -4962,8 +5290,11 @@
       <c r="H107" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I107" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>3</v>
       </c>
@@ -4988,8 +5319,11 @@
       <c r="H108" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I108" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>3</v>
       </c>
@@ -5014,8 +5348,11 @@
       <c r="H109" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I109" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>3</v>
       </c>
@@ -5040,8 +5377,11 @@
       <c r="H110" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I110" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>3</v>
       </c>
@@ -5066,8 +5406,11 @@
       <c r="H111" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I111" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>3</v>
       </c>
@@ -5092,8 +5435,11 @@
       <c r="H112" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I112" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>3</v>
       </c>
@@ -5118,8 +5464,11 @@
       <c r="H113" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I113" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>3</v>
       </c>
@@ -5144,8 +5493,11 @@
       <c r="H114" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I114" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>3</v>
       </c>
@@ -5170,8 +5522,11 @@
       <c r="H115" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I115" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>3</v>
       </c>
@@ -5196,8 +5551,11 @@
       <c r="H116" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I116" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>3</v>
       </c>
@@ -5222,8 +5580,11 @@
       <c r="H117" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I117" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>3</v>
       </c>
@@ -5248,8 +5609,11 @@
       <c r="H118" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I118" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>3</v>
       </c>
@@ -5274,8 +5638,11 @@
       <c r="H119" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I119" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>3</v>
       </c>
@@ -5300,8 +5667,11 @@
       <c r="H120" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I120" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>3</v>
       </c>
@@ -5326,8 +5696,11 @@
       <c r="H121" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I121" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>3</v>
       </c>
@@ -5352,8 +5725,11 @@
       <c r="H122" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I122" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>3</v>
       </c>
@@ -5378,8 +5754,11 @@
       <c r="H123" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I123" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>3</v>
       </c>
@@ -5404,8 +5783,11 @@
       <c r="H124" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I124" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>3</v>
       </c>
@@ -5430,8 +5812,11 @@
       <c r="H125" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I125" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>3</v>
       </c>
@@ -5456,8 +5841,11 @@
       <c r="H126" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I126" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>3</v>
       </c>
@@ -5482,8 +5870,11 @@
       <c r="H127" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I127" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>3</v>
       </c>
@@ -5508,8 +5899,11 @@
       <c r="H128" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I128" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>3</v>
       </c>
@@ -5534,8 +5928,11 @@
       <c r="H129" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I129" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>3</v>
       </c>
@@ -5560,8 +5957,11 @@
       <c r="H130" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I130" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>3</v>
       </c>
@@ -5586,8 +5986,11 @@
       <c r="H131" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I131" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>3</v>
       </c>
@@ -5612,8 +6015,11 @@
       <c r="H132" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I132" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>3</v>
       </c>
@@ -5638,8 +6044,11 @@
       <c r="H133" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I133" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>3</v>
       </c>
@@ -5664,8 +6073,11 @@
       <c r="H134" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I134" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>3</v>
       </c>
@@ -5690,8 +6102,11 @@
       <c r="H135" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I135" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>3</v>
       </c>
@@ -5716,8 +6131,11 @@
       <c r="H136" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I136" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>3</v>
       </c>
@@ -5742,8 +6160,11 @@
       <c r="H137" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I137" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>3</v>
       </c>
@@ -5768,8 +6189,11 @@
       <c r="H138" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I138" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>3</v>
       </c>
@@ -5794,8 +6218,11 @@
       <c r="H139" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I139" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>3</v>
       </c>
@@ -5820,8 +6247,11 @@
       <c r="H140" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I140" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>3</v>
       </c>
@@ -5846,8 +6276,11 @@
       <c r="H141" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I141" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>3</v>
       </c>
@@ -5872,8 +6305,11 @@
       <c r="H142" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I142" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>3</v>
       </c>
@@ -5898,8 +6334,11 @@
       <c r="H143" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I143" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>3</v>
       </c>
@@ -5924,8 +6363,11 @@
       <c r="H144" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I144" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>3</v>
       </c>
@@ -5950,8 +6392,11 @@
       <c r="H145" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I145" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>3</v>
       </c>
@@ -5976,8 +6421,11 @@
       <c r="H146" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I146" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>3</v>
       </c>
@@ -6002,8 +6450,11 @@
       <c r="H147" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I147" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>3</v>
       </c>
@@ -6028,8 +6479,11 @@
       <c r="H148" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I148" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>3</v>
       </c>
@@ -6054,8 +6508,11 @@
       <c r="H149" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I149" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>3</v>
       </c>
@@ -6080,8 +6537,11 @@
       <c r="H150" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I150" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>3</v>
       </c>
@@ -6106,8 +6566,11 @@
       <c r="H151" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I151" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>3</v>
       </c>
@@ -6132,8 +6595,11 @@
       <c r="H152" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I152" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>3</v>
       </c>
@@ -6158,8 +6624,11 @@
       <c r="H153" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I153" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>3</v>
       </c>
@@ -6184,8 +6653,11 @@
       <c r="H154" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I154" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>3</v>
       </c>
@@ -6210,8 +6682,11 @@
       <c r="H155" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I155" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>3</v>
       </c>
@@ -6236,8 +6711,11 @@
       <c r="H156" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I156" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>3</v>
       </c>
@@ -6262,8 +6740,11 @@
       <c r="H157" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I157" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>3</v>
       </c>
@@ -6288,8 +6769,11 @@
       <c r="H158" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I158" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>3</v>
       </c>
@@ -6314,8 +6798,11 @@
       <c r="H159" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I159" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>3</v>
       </c>
@@ -6340,8 +6827,11 @@
       <c r="H160" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I160" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>3</v>
       </c>
@@ -6366,8 +6856,11 @@
       <c r="H161" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I161" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>3</v>
       </c>
@@ -6392,8 +6885,11 @@
       <c r="H162" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I162" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>3</v>
       </c>
@@ -6418,8 +6914,11 @@
       <c r="H163" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I163" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>3</v>
       </c>
@@ -6444,8 +6943,11 @@
       <c r="H164" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I164" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>3</v>
       </c>
@@ -6470,8 +6972,11 @@
       <c r="H165" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I165" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>4</v>
       </c>
@@ -6493,8 +6998,11 @@
       <c r="G166">
         <v>50</v>
       </c>
-    </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I166" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>4</v>
       </c>
@@ -6516,8 +7024,11 @@
       <c r="G167">
         <v>500</v>
       </c>
-    </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I167" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>4</v>
       </c>
@@ -6539,8 +7050,11 @@
       <c r="G168">
         <v>1500</v>
       </c>
-    </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I168" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>4</v>
       </c>
@@ -6562,8 +7076,11 @@
       <c r="G169">
         <v>2500</v>
       </c>
-    </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I169" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>4</v>
       </c>
@@ -6585,8 +7102,11 @@
       <c r="G170">
         <v>50</v>
       </c>
-    </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I170" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>4</v>
       </c>
@@ -6608,8 +7128,11 @@
       <c r="G171">
         <v>1000</v>
       </c>
-    </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I171" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>4</v>
       </c>
@@ -6631,8 +7154,11 @@
       <c r="G172">
         <v>3000</v>
       </c>
-    </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I172" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>4</v>
       </c>
@@ -6654,8 +7180,11 @@
       <c r="G173">
         <v>5000</v>
       </c>
-    </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I173" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>4</v>
       </c>
@@ -6677,8 +7206,11 @@
       <c r="G174">
         <v>50</v>
       </c>
-    </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I174" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>4</v>
       </c>
@@ -6700,8 +7232,11 @@
       <c r="G175">
         <v>1500</v>
       </c>
-    </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I175" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>4</v>
       </c>
@@ -6723,8 +7258,11 @@
       <c r="G176">
         <v>4500</v>
       </c>
-    </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I176" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>4</v>
       </c>
@@ -6746,8 +7284,11 @@
       <c r="G177">
         <v>7500</v>
       </c>
-    </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I177" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>4</v>
       </c>
@@ -6769,8 +7310,11 @@
       <c r="G178">
         <v>50</v>
       </c>
-    </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I178" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>4</v>
       </c>
@@ -6792,8 +7336,11 @@
       <c r="G179">
         <v>1000</v>
       </c>
-    </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I179" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>4</v>
       </c>
@@ -6815,8 +7362,11 @@
       <c r="G180">
         <v>3000</v>
       </c>
-    </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I180" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>4</v>
       </c>
@@ -6838,8 +7388,11 @@
       <c r="G181">
         <v>5000</v>
       </c>
-    </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I181" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>4</v>
       </c>
@@ -6861,8 +7414,11 @@
       <c r="G182">
         <v>50</v>
       </c>
-    </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I182" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>4</v>
       </c>
@@ -6884,8 +7440,11 @@
       <c r="G183">
         <v>1000</v>
       </c>
-    </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I183" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>4</v>
       </c>
@@ -6907,8 +7466,11 @@
       <c r="G184">
         <v>3000</v>
       </c>
-    </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I184" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>4</v>
       </c>
@@ -6930,8 +7492,11 @@
       <c r="G185">
         <v>5000</v>
       </c>
-    </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I185" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>4</v>
       </c>
@@ -6954,8 +7519,11 @@
       <c r="G186">
         <v>50</v>
       </c>
-    </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I186" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>4</v>
       </c>
@@ -6978,8 +7546,11 @@
       <c r="G187">
         <v>500</v>
       </c>
-    </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I187" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>4</v>
       </c>
@@ -7002,8 +7573,11 @@
       <c r="G188">
         <v>1500</v>
       </c>
-    </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I188" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>4</v>
       </c>
@@ -7026,8 +7600,11 @@
       <c r="G189">
         <v>2500</v>
       </c>
-    </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I189" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>4</v>
       </c>
@@ -7050,8 +7627,11 @@
       <c r="G190">
         <v>50</v>
       </c>
-    </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I190" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>4</v>
       </c>
@@ -7074,8 +7654,11 @@
       <c r="G191">
         <v>1500</v>
       </c>
-    </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I191" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>4</v>
       </c>
@@ -7098,8 +7681,11 @@
       <c r="G192">
         <v>4500</v>
       </c>
-    </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I192" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>4</v>
       </c>
@@ -7122,8 +7708,11 @@
       <c r="G193">
         <v>7500</v>
       </c>
-    </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I193" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>4</v>
       </c>
@@ -7146,8 +7735,11 @@
       <c r="G194">
         <v>50</v>
       </c>
-    </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I194" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>4</v>
       </c>
@@ -7170,8 +7762,11 @@
       <c r="G195">
         <v>1000</v>
       </c>
-    </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I195" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>4</v>
       </c>
@@ -7194,8 +7789,11 @@
       <c r="G196">
         <v>3000</v>
       </c>
-    </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I196" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>4</v>
       </c>
@@ -7218,8 +7816,11 @@
       <c r="G197">
         <v>5000</v>
       </c>
-    </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I197" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>4</v>
       </c>
@@ -7242,8 +7843,11 @@
       <c r="G198">
         <v>50</v>
       </c>
-    </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I198" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>4</v>
       </c>
@@ -7266,8 +7870,11 @@
       <c r="G199">
         <v>1000</v>
       </c>
-    </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I199" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>4</v>
       </c>
@@ -7290,8 +7897,11 @@
       <c r="G200">
         <v>3000</v>
       </c>
-    </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I200" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>4</v>
       </c>
@@ -7314,8 +7924,11 @@
       <c r="G201">
         <v>5000</v>
       </c>
-    </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I201" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>4</v>
       </c>
@@ -7338,8 +7951,11 @@
       <c r="G202">
         <v>50</v>
       </c>
-    </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I202" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>4</v>
       </c>
@@ -7362,8 +7978,11 @@
       <c r="G203">
         <v>1500</v>
       </c>
-    </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I203" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>4</v>
       </c>
@@ -7386,8 +8005,11 @@
       <c r="G204">
         <v>4500</v>
       </c>
-    </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I204" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>4</v>
       </c>
@@ -7410,8 +8032,11 @@
       <c r="G205">
         <v>7500</v>
       </c>
-    </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I205" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>4</v>
       </c>
@@ -7434,8 +8059,11 @@
       <c r="G206">
         <v>50</v>
       </c>
-    </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I206" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>4</v>
       </c>
@@ -7458,8 +8086,11 @@
       <c r="G207">
         <v>500</v>
       </c>
-    </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I207" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>4</v>
       </c>
@@ -7482,8 +8113,11 @@
       <c r="G208">
         <v>1500</v>
       </c>
-    </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I208" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>4</v>
       </c>
@@ -7506,8 +8140,11 @@
       <c r="G209">
         <v>2500</v>
       </c>
-    </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I209" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>4</v>
       </c>
@@ -7530,8 +8167,11 @@
       <c r="G210">
         <v>50</v>
       </c>
-    </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I210" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>4</v>
       </c>
@@ -7554,8 +8194,11 @@
       <c r="G211">
         <v>1000</v>
       </c>
-    </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I211" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="212" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>4</v>
       </c>
@@ -7578,8 +8221,11 @@
       <c r="G212">
         <v>3000</v>
       </c>
-    </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I212" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>4</v>
       </c>
@@ -7602,8 +8248,11 @@
       <c r="G213">
         <v>5000</v>
       </c>
-    </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I213" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="214" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>4</v>
       </c>
@@ -7626,8 +8275,11 @@
       <c r="G214">
         <v>50</v>
       </c>
-    </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I214" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>4</v>
       </c>
@@ -7650,8 +8302,11 @@
       <c r="G215">
         <v>1000</v>
       </c>
-    </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I215" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="216" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>4</v>
       </c>
@@ -7674,8 +8329,11 @@
       <c r="G216">
         <v>3000</v>
       </c>
-    </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I216" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="217" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>4</v>
       </c>
@@ -7698,8 +8356,11 @@
       <c r="G217">
         <v>5000</v>
       </c>
-    </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I217" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="218" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>4</v>
       </c>
@@ -7722,8 +8383,11 @@
       <c r="G218">
         <v>50</v>
       </c>
-    </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I218" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="219" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>4</v>
       </c>
@@ -7746,8 +8410,11 @@
       <c r="G219">
         <v>500</v>
       </c>
-    </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I219" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="220" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>4</v>
       </c>
@@ -7770,8 +8437,11 @@
       <c r="G220">
         <v>1500</v>
       </c>
-    </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I220" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="221" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>4</v>
       </c>
@@ -7794,8 +8464,11 @@
       <c r="G221">
         <v>2500</v>
       </c>
-    </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I221" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="222" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>4</v>
       </c>
@@ -7818,8 +8491,11 @@
       <c r="G222">
         <v>50</v>
       </c>
-    </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I222" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>4</v>
       </c>
@@ -7842,8 +8518,11 @@
       <c r="G223">
         <v>1000</v>
       </c>
-    </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I223" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="224" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>4</v>
       </c>
@@ -7866,8 +8545,11 @@
       <c r="G224">
         <v>3000</v>
       </c>
-    </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I224" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="225" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>4</v>
       </c>
@@ -7890,8 +8572,11 @@
       <c r="G225">
         <v>5000</v>
       </c>
-    </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I225" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="226" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>4</v>
       </c>
@@ -7914,8 +8599,11 @@
       <c r="G226">
         <v>50</v>
       </c>
-    </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I226" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="227" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>4</v>
       </c>
@@ -7938,8 +8626,11 @@
       <c r="G227">
         <v>1000</v>
       </c>
-    </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I227" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="228" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>4</v>
       </c>
@@ -7962,8 +8653,11 @@
       <c r="G228">
         <v>3000</v>
       </c>
-    </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I228" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="229" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>4</v>
       </c>
@@ -7986,8 +8680,11 @@
       <c r="G229">
         <v>5000</v>
       </c>
-    </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I229" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="230" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>4</v>
       </c>
@@ -8010,8 +8707,11 @@
       <c r="G230">
         <v>50</v>
       </c>
-    </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I230" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="231" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>4</v>
       </c>
@@ -8034,8 +8734,11 @@
       <c r="G231">
         <v>500</v>
       </c>
-    </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I231" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="232" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>4</v>
       </c>
@@ -8058,8 +8761,11 @@
       <c r="G232">
         <v>1500</v>
       </c>
-    </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I232" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="233" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>4</v>
       </c>
@@ -8082,8 +8788,11 @@
       <c r="G233">
         <v>2500</v>
       </c>
-    </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I233" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="234" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>4</v>
       </c>
@@ -8106,8 +8815,11 @@
       <c r="G234">
         <v>50</v>
       </c>
-    </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I234" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="235" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>4</v>
       </c>
@@ -8130,8 +8842,11 @@
       <c r="G235">
         <v>1000</v>
       </c>
-    </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I235" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>4</v>
       </c>
@@ -8154,8 +8869,11 @@
       <c r="G236">
         <v>3000</v>
       </c>
-    </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I236" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>4</v>
       </c>
@@ -8178,8 +8896,11 @@
       <c r="G237">
         <v>5000</v>
       </c>
-    </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I237" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>4</v>
       </c>
@@ -8202,8 +8923,11 @@
       <c r="G238">
         <v>50</v>
       </c>
-    </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I238" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="239" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>4</v>
       </c>
@@ -8226,8 +8950,11 @@
       <c r="G239">
         <v>1000</v>
       </c>
-    </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I239" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="240" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>4</v>
       </c>
@@ -8250,8 +8977,11 @@
       <c r="G240">
         <v>3000</v>
       </c>
-    </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I240" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="241" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>4</v>
       </c>
@@ -8274,8 +9004,11 @@
       <c r="G241">
         <v>5000</v>
       </c>
-    </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I241" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="242" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>4</v>
       </c>
@@ -8298,8 +9031,11 @@
       <c r="G242">
         <v>50</v>
       </c>
-    </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I242" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="243" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>4</v>
       </c>
@@ -8322,8 +9058,11 @@
       <c r="G243">
         <v>500</v>
       </c>
-    </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I243" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="244" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>4</v>
       </c>
@@ -8346,8 +9085,11 @@
       <c r="G244">
         <v>1500</v>
       </c>
-    </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I244" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="245" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>4</v>
       </c>
@@ -8370,8 +9112,11 @@
       <c r="G245">
         <v>2500</v>
       </c>
-    </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I245" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="246" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>4</v>
       </c>
@@ -8394,8 +9139,11 @@
       <c r="G246">
         <v>50</v>
       </c>
-    </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I246" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="247" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>4</v>
       </c>
@@ -8418,8 +9166,11 @@
       <c r="G247">
         <v>1000</v>
       </c>
-    </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I247" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="248" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>4</v>
       </c>
@@ -8442,8 +9193,11 @@
       <c r="G248">
         <v>3000</v>
       </c>
-    </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I248" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="249" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>4</v>
       </c>
@@ -8466,8 +9220,11 @@
       <c r="G249">
         <v>5000</v>
       </c>
-    </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I249" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="250" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>4</v>
       </c>
@@ -8490,8 +9247,11 @@
       <c r="G250">
         <v>50</v>
       </c>
-    </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I250" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="251" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>4</v>
       </c>
@@ -8514,8 +9274,11 @@
       <c r="G251">
         <v>500</v>
       </c>
-    </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I251" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="252" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>4</v>
       </c>
@@ -8538,8 +9301,11 @@
       <c r="G252">
         <v>1500</v>
       </c>
-    </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I252" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="253" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>4</v>
       </c>
@@ -8562,8 +9328,11 @@
       <c r="G253">
         <v>2500</v>
       </c>
-    </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I253" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="254" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>4</v>
       </c>
@@ -8586,8 +9355,11 @@
       <c r="G254">
         <v>50</v>
       </c>
-    </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I254" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="255" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>4</v>
       </c>
@@ -8610,8 +9382,11 @@
       <c r="G255">
         <v>1000</v>
       </c>
-    </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I255" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="256" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>4</v>
       </c>
@@ -8634,8 +9409,11 @@
       <c r="G256">
         <v>3000</v>
       </c>
-    </row>
-    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I256" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="257" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>4</v>
       </c>
@@ -8658,8 +9436,11 @@
       <c r="G257">
         <v>5000</v>
       </c>
-    </row>
-    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I257" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="258" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>4</v>
       </c>
@@ -8682,8 +9463,11 @@
       <c r="G258">
         <v>50</v>
       </c>
-    </row>
-    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I258" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="259" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>4</v>
       </c>
@@ -8706,8 +9490,11 @@
       <c r="G259">
         <v>500</v>
       </c>
-    </row>
-    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I259" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="260" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>4</v>
       </c>
@@ -8730,8 +9517,11 @@
       <c r="G260">
         <v>1500</v>
       </c>
-    </row>
-    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I260" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="261" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>4</v>
       </c>
@@ -8754,8 +9544,11 @@
       <c r="G261">
         <v>2500</v>
       </c>
-    </row>
-    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I261" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="262" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>4</v>
       </c>
@@ -8778,8 +9571,11 @@
       <c r="G262">
         <v>50</v>
       </c>
-    </row>
-    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I262" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="263" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>4</v>
       </c>
@@ -8802,8 +9598,11 @@
       <c r="G263">
         <v>1000</v>
       </c>
-    </row>
-    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I263" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="264" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>4</v>
       </c>
@@ -8826,8 +9625,11 @@
       <c r="G264">
         <v>3000</v>
       </c>
-    </row>
-    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I264" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="265" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>4</v>
       </c>
@@ -8850,8 +9652,11 @@
       <c r="G265">
         <v>5000</v>
       </c>
-    </row>
-    <row r="266" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I265" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="266" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>3</v>
       </c>
@@ -8876,8 +9681,11 @@
       <c r="H266" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="267" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I266" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="267" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>3</v>
       </c>
@@ -8902,8 +9710,11 @@
       <c r="H267" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="268" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I267" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="268" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>3</v>
       </c>
@@ -8928,8 +9739,11 @@
       <c r="H268" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="269" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I268" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="269" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>3</v>
       </c>
@@ -8954,8 +9768,11 @@
       <c r="H269" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="270" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I269" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="270" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>3</v>
       </c>
@@ -8980,8 +9797,11 @@
       <c r="H270" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="271" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I270" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="271" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>3</v>
       </c>
@@ -9006,8 +9826,11 @@
       <c r="H271" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="272" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I271" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="272" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>3</v>
       </c>
@@ -9032,8 +9855,11 @@
       <c r="H272" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="273" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I272" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="273" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>3</v>
       </c>
@@ -9058,8 +9884,11 @@
       <c r="H273" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="274" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I273" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="274" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>4</v>
       </c>
@@ -9082,8 +9911,11 @@
       <c r="G274">
         <v>50</v>
       </c>
-    </row>
-    <row r="275" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I274" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="275" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>4</v>
       </c>
@@ -9103,8 +9935,11 @@
         <f t="shared" si="3"/>
         <v>Low</v>
       </c>
-    </row>
-    <row r="276" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I275" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="276" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>4</v>
       </c>
@@ -9127,8 +9962,11 @@
       <c r="G276">
         <v>500</v>
       </c>
-    </row>
-    <row r="277" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I276" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="277" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>4</v>
       </c>
@@ -9150,6 +9988,9 @@
       </c>
       <c r="G277">
         <v>1000</v>
+      </c>
+      <c r="I277" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added fall chinook lgr figures and moved pHOS graphic inset
</commit_message>
<xml_diff>
--- a/data/input/mgt_targets.xlsx
+++ b/data/input/mgt_targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\SRAFS\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A6B8FA6-D8D8-4AD3-BDB9-86790E19BC51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5083F429-58AA-4D18-864B-9F86240AD7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Goals and Thresholds" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Notes" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">pop_targets!$A$1:$H$265</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">pop_targets!$A$1:$I$277</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">targets!$A$1:$H$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2303" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2310" uniqueCount="111">
   <si>
     <t xml:space="preserve">Total </t>
   </si>
@@ -492,6 +492,9 @@
   </si>
   <si>
     <t>Extant</t>
+  </si>
+  <si>
+    <t>Was - 3614; Quasi-Extinction Threshold (QET) of 50 times number of populations upstream of Lower Granite Dam.  U.S. vs Oregon Production Advisory Committee Broodstock Needs Table</t>
   </si>
 </sst>
 </file>
@@ -1287,8 +1290,8 @@
     <col min="3" max="3" width="18.7109375" customWidth="1"/>
     <col min="4" max="4" width="17.7109375" customWidth="1"/>
     <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" customWidth="1"/>
-    <col min="7" max="7" width="24.7109375" customWidth="1"/>
+    <col min="6" max="6" width="34.5703125" customWidth="1"/>
+    <col min="7" max="7" width="46.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1497,6 +1500,9 @@
       <c r="F9">
         <v>24800</v>
       </c>
+      <c r="G9" t="s">
+        <v>83</v>
+      </c>
       <c r="H9" t="s">
         <v>39</v>
       </c>
@@ -1518,10 +1524,13 @@
         <v>78</v>
       </c>
       <c r="F10">
-        <v>3614</v>
+        <v>4100</v>
+      </c>
+      <c r="G10" t="s">
+        <v>84</v>
       </c>
       <c r="H10" t="s">
-        <v>37</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1543,6 +1552,9 @@
       <c r="F11">
         <v>43000</v>
       </c>
+      <c r="G11" t="s">
+        <v>81</v>
+      </c>
       <c r="H11" t="s">
         <v>39</v>
       </c>
@@ -1566,6 +1578,9 @@
       <c r="F12">
         <v>50</v>
       </c>
+      <c r="G12" t="s">
+        <v>41</v>
+      </c>
       <c r="H12" t="s">
         <v>37</v>
       </c>
@@ -1589,6 +1604,9 @@
       <c r="F13">
         <v>18200</v>
       </c>
+      <c r="G13" t="s">
+        <v>82</v>
+      </c>
       <c r="H13" t="s">
         <v>39</v>
       </c>
@@ -1612,6 +1630,9 @@
       <c r="F14">
         <v>5300</v>
       </c>
+      <c r="G14" t="s">
+        <v>86</v>
+      </c>
       <c r="H14" t="s">
         <v>40</v>
       </c>
@@ -1635,6 +1656,9 @@
       <c r="F15">
         <v>11700</v>
       </c>
+      <c r="G15" t="s">
+        <v>85</v>
+      </c>
       <c r="H15" t="s">
         <v>40</v>
       </c>
@@ -2165,6 +2189,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H36" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H36">
     <sortCondition ref="A2:A36"/>
     <sortCondition ref="D2:D36"/>

</xml_diff>